<commit_message>
Add OCR for scans and photos
</commit_message>
<xml_diff>
--- a/invoices.xlsx
+++ b/invoices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -636,6 +636,132 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>photo3.jpg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BW/2024/0562</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5 June 2024</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Brightway Consulting Ltd</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>£2,850.00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>£570.00</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>£3,420.00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>photo4.jpg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV-20240911</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sep 11, 2024</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sunrise Bakery</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>$531.00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>$43.81</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>$574.81</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>scan2.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2024-0187</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>14.03.2024</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GreenLeaf Studio GmbH</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1,050.00 €</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>199.50 €</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1,249.50 €</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>